<commit_message>
Update Excel comparison report with all requested detailed columns
</commit_message>
<xml_diff>
--- a/results/model_comparison_report.xlsx
+++ b/results/model_comparison_report.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="All Groups Evaluation" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="300 Groups Evaluation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="50 Groups Evaluation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Master Model Comparison" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="All Groups Evaluation" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="300 Groups Evaluation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="50 Groups Evaluation" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,10 +20,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="+0.00%;-0.00%;0.00%"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -84,6 +86,17 @@
       <color rgb="00375623"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00375623"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -137,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -159,17 +172,29 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="11" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -177,8 +202,14 @@
     <xf numFmtId="2" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -693,31 +724,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:L25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="107" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="59" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>All Groups Evaluation Detailed Results Table</t>
+          <t>Master Model Comparison Detailed Results Table</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Evaluated on validation period: 2012-08-17 to 2012-10-26</t>
+          <t>Master consolidated model comparisons across all scopes | Validation period: 2012-08-17 to 2012-10-26</t>
         </is>
       </c>
     </row>
@@ -729,40 +763,55 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>WMAE ($)</t>
+          <t>Groups</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>MAE ($)</t>
+          <t>Model Parameters</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>RMSE ($)</t>
+          <t>WMAE</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>MAPE (%)</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>sMAPE (%)</t>
+          <t>RMSE</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
+          <t>sMAPE</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
           <t>Runtime</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Improvement vs Baseline</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Fit Success</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
@@ -774,313 +823,1006 @@
           <t>Holt-Winters</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
         <v>1427.69</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="F5" s="13" t="n">
         <v>1422.5</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="G5" s="13" t="n">
         <v>3130.43</v>
       </c>
-      <c r="F5" s="12" t="n">
-        <v>2.8975</v>
-      </c>
-      <c r="G5" s="12" t="n">
+      <c r="H5" s="14" t="n">
         <v>23.71</v>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>33.4 min (2006s)</t>
         </is>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="J5" s="15" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>SARIMA(1,1,0)x(0,1,1,52)</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="n">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="n">
         <v>1494.19</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="F6" s="19" t="n">
         <v>1495.93</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="G6" s="19" t="n">
         <v>3189.19</v>
       </c>
-      <c r="F6" s="16" t="n">
-        <v>4.4387</v>
-      </c>
-      <c r="G6" s="16" t="n">
+      <c r="H6" s="20" t="n">
         <v>24.42</v>
       </c>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>57.3 min (3436s)</t>
         </is>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="J6" s="21" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L6" s="17" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Seasonal Naive (Subset)</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="n">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on eligible groups with &gt;= 104 weeks history)</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>1714.9</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="F7" s="19" t="n">
         <v>1689.93</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="G7" s="19" t="n">
         <v>3638.77</v>
       </c>
-      <c r="F7" s="16" t="n">
-        <v>23.0952</v>
-      </c>
-      <c r="G7" s="16" t="n">
+      <c r="H7" s="20" t="n">
         <v>23.35</v>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>0.16s</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="J7" s="21" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Seasonal Naive (Full)</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Baseline Model</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="n">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on all 3,084 groups)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="n">
         <v>1723.13</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="F8" s="19" t="n">
         <v>1698.02</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="G8" s="19" t="n">
         <v>3658.17</v>
       </c>
-      <c r="F8" s="16" t="n">
-        <v>24.0012</v>
-      </c>
-      <c r="G8" s="16" t="n">
+      <c r="H8" s="20" t="n">
         <v>23.46</v>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>0.13s</t>
         </is>
       </c>
-      <c r="I8" s="17" t="n">
+      <c r="J8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Simple Exp Smoothing (SES)</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="n">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
         <v>2143.17</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="F9" s="19" t="n">
         <v>2156.63</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="G9" s="19" t="n">
         <v>4800.22</v>
       </c>
-      <c r="F9" s="16" t="n">
-        <v>2.362</v>
-      </c>
-      <c r="G9" s="16" t="n">
+      <c r="H9" s="20" t="n">
         <v>26.41</v>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>33.8 min (2029s)</t>
         </is>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="J9" s="23" t="n">
+        <v>-24.38</v>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Holt's Linear Trend</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="n">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="n">
         <v>2155.95</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="F10" s="19" t="n">
         <v>2166.05</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="G10" s="19" t="n">
         <v>5261.12</v>
       </c>
-      <c r="F10" s="16" t="n">
-        <v>2.5483</v>
-      </c>
-      <c r="G10" s="16" t="n">
+      <c r="H10" s="20" t="n">
         <v>27.01</v>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>32.9 min (1974s)</t>
         </is>
       </c>
-      <c r="I10" s="17" t="n">
+      <c r="J10" s="23" t="n">
+        <v>-25.12</v>
+      </c>
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>ARIMA(1,1,1)</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="n">
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="n">
         <v>2210.61</v>
       </c>
-      <c r="D11" s="15" t="n">
+      <c r="F11" s="19" t="n">
         <v>2197.86</v>
       </c>
-      <c r="E11" s="15" t="n">
+      <c r="G11" s="19" t="n">
         <v>4920.17</v>
       </c>
-      <c r="F11" s="16" t="n">
-        <v>4.4993</v>
-      </c>
-      <c r="G11" s="16" t="n">
+      <c r="H11" s="20" t="n">
         <v>26.33</v>
       </c>
-      <c r="H11" s="17" t="inlineStr">
+      <c r="I11" s="17" t="inlineStr">
         <is>
           <t>35.5 min (2131s)</t>
         </is>
       </c>
-      <c r="I11" s="17" t="n">
+      <c r="J11" s="23" t="n">
+        <v>-28.29</v>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L11" s="17" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Naive</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>Baseline Model</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="n">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>period=1 (uses final week's sales value as static forecast)</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="n">
         <v>2241.28</v>
       </c>
-      <c r="D12" s="15" t="n">
+      <c r="F12" s="19" t="n">
         <v>2308.47</v>
       </c>
-      <c r="E12" s="15" t="n">
+      <c r="G12" s="19" t="n">
         <v>5080.3</v>
       </c>
-      <c r="F12" s="16" t="n">
-        <v>4.1667</v>
-      </c>
-      <c r="G12" s="16" t="n">
+      <c r="H12" s="20" t="n">
         <v>28.25</v>
       </c>
-      <c r="H12" s="17" t="inlineStr">
+      <c r="I12" s="17" t="inlineStr">
         <is>
           <t>0.16s</t>
         </is>
       </c>
-      <c r="I12" s="17" t="n">
+      <c r="J12" s="23" t="n">
+        <v>-30.07</v>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L12" s="17" t="n">
         <v>8</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Historical Mean</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>Baseline Model</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="n">
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>static average calculated per group</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="n">
         <v>2524.38</v>
       </c>
-      <c r="D13" s="15" t="n">
+      <c r="F13" s="19" t="n">
         <v>2425.44</v>
       </c>
-      <c r="E13" s="15" t="n">
+      <c r="G13" s="19" t="n">
         <v>4953.47</v>
       </c>
-      <c r="F13" s="16" t="n">
-        <v>28.0084</v>
-      </c>
-      <c r="G13" s="16" t="n">
+      <c r="H13" s="20" t="n">
         <v>29.2</v>
       </c>
-      <c r="H13" s="17" t="inlineStr">
+      <c r="I13" s="17" t="inlineStr">
         <is>
           <t>0.03s</t>
         </is>
       </c>
-      <c r="I13" s="17" t="n">
+      <c r="J13" s="23" t="n">
+        <v>-46.5</v>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Holt-Winters</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="n">
+        <v>4538.4</v>
+      </c>
+      <c r="F14" s="13" t="n">
+        <v>4557.37</v>
+      </c>
+      <c r="G14" s="13" t="n">
+        <v>6930.41</v>
+      </c>
+      <c r="H14" s="14" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="I14" s="11" t="inlineStr">
+        <is>
+          <t>17.2s</t>
+        </is>
+      </c>
+      <c r="J14" s="15" t="n">
+        <v>23.97</v>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L14" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>4721.37</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>4761.32</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>7166.81</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>168.4s</t>
+        </is>
+      </c>
+      <c r="J15" s="21" t="n">
+        <v>20.91</v>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L15" s="17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Simple Exp Smoothing (SES)</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>5842.2</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>5639.89</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>7977.69</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>29.5s</t>
+        </is>
+      </c>
+      <c r="J16" s="21" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L16" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Holt's Linear Trend</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>5882.53</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>5679.11</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>8026.3</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>22.7s</t>
+        </is>
+      </c>
+      <c r="J17" s="21" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L17" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>ARIMA(1,1,1)</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>5915.22</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>5626.12</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>7813.31</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>8.7s</t>
+        </is>
+      </c>
+      <c r="J18" s="21" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="K18" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L18" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal Naive</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on all 300 high-volume groups)</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>5969.34</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>5856.3</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>8924.129999999999</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>0.04s</t>
+        </is>
+      </c>
+      <c r="J19" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L19" s="17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Holt-Winters</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>6838.89</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>6753.86</v>
+      </c>
+      <c r="G20" s="13" t="n">
+        <v>9852.280000000001</v>
+      </c>
+      <c r="H20" s="14" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I20" s="11" t="inlineStr">
+        <is>
+          <t>1.37s</t>
+        </is>
+      </c>
+      <c r="J20" s="15" t="n">
+        <v>32.65</v>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L20" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>7375.57</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>7465.79</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>11072.19</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>62.2s</t>
+        </is>
+      </c>
+      <c r="J21" s="21" t="n">
+        <v>27.37</v>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L21" s="17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>ARIMA(1,1,1)</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>9148.290000000001</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>8670.959999999999</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>11257.67</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>0.80s</t>
+        </is>
+      </c>
+      <c r="J22" s="21" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L22" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>Simple Exp Smoothing (SES)</t>
+        </is>
+      </c>
+      <c r="B23" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D23" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E23" s="19" t="n">
+        <v>9166.110000000001</v>
+      </c>
+      <c r="F23" s="19" t="n">
+        <v>8779.459999999999</v>
+      </c>
+      <c r="G23" s="19" t="n">
+        <v>11333.78</v>
+      </c>
+      <c r="H23" s="20" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="I23" s="17" t="inlineStr">
+        <is>
+          <t>1.99s</t>
+        </is>
+      </c>
+      <c r="J23" s="21" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="K23" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L23" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>Holt's Linear Trend</t>
+        </is>
+      </c>
+      <c r="B24" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C24" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D24" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E24" s="19" t="n">
+        <v>9327.07</v>
+      </c>
+      <c r="F24" s="19" t="n">
+        <v>8889.629999999999</v>
+      </c>
+      <c r="G24" s="19" t="n">
+        <v>11473.64</v>
+      </c>
+      <c r="H24" s="20" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="I24" s="17" t="inlineStr">
+        <is>
+          <t>0.46s</t>
+        </is>
+      </c>
+      <c r="J24" s="21" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L24" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal Naive</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on all 50 high-volume groups)</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>10154.41</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>9921.17</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>14704.32</v>
+      </c>
+      <c r="H25" s="20" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>0.01s</t>
+        </is>
+      </c>
+      <c r="J25" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L25" s="17" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1094,31 +1836,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="107" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="59" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>300 Groups Evaluation Detailed Results Table</t>
+          <t>All Groups Evaluation Detailed Results Table</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Evaluated on validation period: 2012-08-17 to 2012-10-26</t>
+          <t>Evaluated on all 3,084 Store-Department validation groups | Validation period: 2012-08-17 to 2012-10-26</t>
         </is>
       </c>
     </row>
@@ -1130,40 +1875,55 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>WMAE ($)</t>
+          <t>Groups</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>MAE ($)</t>
+          <t>Model Parameters</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>RMSE ($)</t>
+          <t>WMAE</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>MAPE (%)</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>sMAPE (%)</t>
+          <t>RMSE</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
+          <t>sMAPE</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
           <t>Runtime</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Improvement vs Baseline</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Fit Success</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
@@ -1175,208 +1935,430 @@
           <t>Holt-Winters</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>4538.4</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>4557.37</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>6930.41</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>7.3004</v>
-      </c>
-      <c r="G5" s="12" t="n">
-        <v>7.49</v>
-      </c>
-      <c r="H5" s="13" t="inlineStr">
-        <is>
-          <t>17.2s</t>
-        </is>
-      </c>
-      <c r="I5" s="13" t="n">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>1427.69</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>1422.5</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>3130.43</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>23.71</v>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>33.4 min (2006s)</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>SARIMA(1,1,0)x(0,1,1,52)</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="n">
-        <v>4721.37</v>
-      </c>
-      <c r="D6" s="15" t="n">
-        <v>4761.32</v>
-      </c>
-      <c r="E6" s="15" t="n">
-        <v>7166.81</v>
-      </c>
-      <c r="F6" s="16" t="n">
-        <v>7.6114</v>
-      </c>
-      <c r="G6" s="16" t="n">
-        <v>7.82</v>
-      </c>
-      <c r="H6" s="17" t="inlineStr">
-        <is>
-          <t>168.4s</t>
-        </is>
-      </c>
-      <c r="I6" s="17" t="n">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>1494.19</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>1495.93</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>3189.19</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>24.42</v>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>57.3 min (3436s)</t>
+        </is>
+      </c>
+      <c r="J6" s="21" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L6" s="17" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal Naive (Subset)</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on eligible groups with &gt;= 104 weeks history)</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>1714.9</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>1689.93</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>3638.77</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>23.35</v>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>0.16s</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal Naive (Full)</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on all 3,084 groups)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>1723.13</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>1698.02</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>3658.17</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>23.46</v>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="J8" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Simple Exp Smoothing (SES)</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>5842.2</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>5639.89</v>
-      </c>
-      <c r="E7" s="15" t="n">
-        <v>7977.69</v>
-      </c>
-      <c r="F7" s="16" t="n">
-        <v>8.8978</v>
-      </c>
-      <c r="G7" s="16" t="n">
-        <v>8.859999999999999</v>
-      </c>
-      <c r="H7" s="17" t="inlineStr">
-        <is>
-          <t>29.5s</t>
-        </is>
-      </c>
-      <c r="I7" s="17" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>2143.17</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>2156.63</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>4800.22</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>26.41</v>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>33.8 min (2029s)</t>
+        </is>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>-24.38</v>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Holt's Linear Trend</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="n">
-        <v>5882.53</v>
-      </c>
-      <c r="D8" s="15" t="n">
-        <v>5679.11</v>
-      </c>
-      <c r="E8" s="15" t="n">
-        <v>8026.3</v>
-      </c>
-      <c r="F8" s="16" t="n">
-        <v>8.914400000000001</v>
-      </c>
-      <c r="G8" s="16" t="n">
-        <v>8.91</v>
-      </c>
-      <c r="H8" s="17" t="inlineStr">
-        <is>
-          <t>22.7s</t>
-        </is>
-      </c>
-      <c r="I8" s="17" t="n">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>2155.95</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>2166.05</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>5261.12</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>27.01</v>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>32.9 min (1974s)</t>
+        </is>
+      </c>
+      <c r="J10" s="23" t="n">
+        <v>-25.12</v>
+      </c>
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>ARIMA(1,1,1)</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="n">
-        <v>5915.22</v>
-      </c>
-      <c r="D9" s="15" t="n">
-        <v>5626.12</v>
-      </c>
-      <c r="E9" s="15" t="n">
-        <v>7813.31</v>
-      </c>
-      <c r="F9" s="16" t="n">
-        <v>9.122400000000001</v>
-      </c>
-      <c r="G9" s="16" t="n">
-        <v>8.85</v>
-      </c>
-      <c r="H9" s="17" t="inlineStr">
-        <is>
-          <t>8.7s</t>
-        </is>
-      </c>
-      <c r="I9" s="17" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="14" t="inlineStr">
-        <is>
-          <t>Seasonal Naive</t>
-        </is>
-      </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Baseline Model</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="n">
-        <v>5969.34</v>
-      </c>
-      <c r="D10" s="15" t="n">
-        <v>5856.3</v>
-      </c>
-      <c r="E10" s="15" t="n">
-        <v>8924.129999999999</v>
-      </c>
-      <c r="F10" s="16" t="n">
-        <v>9.136100000000001</v>
-      </c>
-      <c r="G10" s="16" t="n">
-        <v>9.07</v>
-      </c>
-      <c r="H10" s="17" t="inlineStr">
-        <is>
-          <t>0.04s</t>
-        </is>
-      </c>
-      <c r="I10" s="17" t="n">
-        <v>6</v>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D11" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E11" s="19" t="n">
+        <v>2210.61</v>
+      </c>
+      <c r="F11" s="19" t="n">
+        <v>2197.86</v>
+      </c>
+      <c r="G11" s="19" t="n">
+        <v>4920.17</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>26.33</v>
+      </c>
+      <c r="I11" s="17" t="inlineStr">
+        <is>
+          <t>35.5 min (2131s)</t>
+        </is>
+      </c>
+      <c r="J11" s="23" t="n">
+        <v>-28.29</v>
+      </c>
+      <c r="K11" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L11" s="17" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Naive</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D12" s="16" t="inlineStr">
+        <is>
+          <t>period=1 (uses final week's sales value as static forecast)</t>
+        </is>
+      </c>
+      <c r="E12" s="19" t="n">
+        <v>2241.28</v>
+      </c>
+      <c r="F12" s="19" t="n">
+        <v>2308.47</v>
+      </c>
+      <c r="G12" s="19" t="n">
+        <v>5080.3</v>
+      </c>
+      <c r="H12" s="20" t="n">
+        <v>28.25</v>
+      </c>
+      <c r="I12" s="17" t="inlineStr">
+        <is>
+          <t>0.16s</t>
+        </is>
+      </c>
+      <c r="J12" s="23" t="n">
+        <v>-30.07</v>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L12" s="17" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="inlineStr">
+        <is>
+          <t>Historical Mean</t>
+        </is>
+      </c>
+      <c r="B13" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D13" s="16" t="inlineStr">
+        <is>
+          <t>static average calculated per group</t>
+        </is>
+      </c>
+      <c r="E13" s="19" t="n">
+        <v>2524.38</v>
+      </c>
+      <c r="F13" s="19" t="n">
+        <v>2425.44</v>
+      </c>
+      <c r="G13" s="19" t="n">
+        <v>4953.47</v>
+      </c>
+      <c r="H13" s="20" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="I13" s="17" t="inlineStr">
+        <is>
+          <t>0.03s</t>
+        </is>
+      </c>
+      <c r="J13" s="23" t="n">
+        <v>-46.5</v>
+      </c>
+      <c r="K13" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L13" s="17" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -1390,31 +2372,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I10"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="107" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>50 Groups Evaluation Detailed Results Table</t>
+          <t>300 Groups Evaluation Detailed Results Table</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>Evaluated on validation period: 2012-08-17 to 2012-10-26</t>
+          <t>Evaluated on 300 high-volume validation groups | Validation period: 2012-08-17 to 2012-10-26</t>
         </is>
       </c>
     </row>
@@ -1426,40 +2411,55 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Scope</t>
         </is>
       </c>
       <c r="C4" s="9" t="inlineStr">
         <is>
-          <t>WMAE ($)</t>
+          <t>Groups</t>
         </is>
       </c>
       <c r="D4" s="9" t="inlineStr">
         <is>
-          <t>MAE ($)</t>
+          <t>Model Parameters</t>
         </is>
       </c>
       <c r="E4" s="9" t="inlineStr">
         <is>
-          <t>RMSE ($)</t>
+          <t>WMAE</t>
         </is>
       </c>
       <c r="F4" s="9" t="inlineStr">
         <is>
-          <t>MAPE (%)</t>
+          <t>MAE</t>
         </is>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
-          <t>sMAPE (%)</t>
+          <t>RMSE</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
         <is>
+          <t>sMAPE</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
           <t>Runtime</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Improvement vs Baseline</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Fit Success</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
@@ -1471,207 +2471,677 @@
           <t>Holt-Winters</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C5" s="11" t="n">
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>4538.4</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>4557.37</v>
+      </c>
+      <c r="G5" s="13" t="n">
+        <v>6930.41</v>
+      </c>
+      <c r="H5" s="14" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>17.2s</t>
+        </is>
+      </c>
+      <c r="J5" s="15" t="n">
+        <v>23.97</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="inlineStr">
+        <is>
+          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+        </is>
+      </c>
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>4721.37</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>4761.32</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>7166.81</v>
+      </c>
+      <c r="H6" s="20" t="n">
+        <v>7.82</v>
+      </c>
+      <c r="I6" s="17" t="inlineStr">
+        <is>
+          <t>168.4s</t>
+        </is>
+      </c>
+      <c r="J6" s="21" t="n">
+        <v>20.91</v>
+      </c>
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L6" s="17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="16" t="inlineStr">
+        <is>
+          <t>Simple Exp Smoothing (SES)</t>
+        </is>
+      </c>
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>5842.2</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>5639.89</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>7977.69</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="I7" s="17" t="inlineStr">
+        <is>
+          <t>29.5s</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="inlineStr">
+        <is>
+          <t>Holt's Linear Trend</t>
+        </is>
+      </c>
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>5882.53</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>5679.11</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>8026.3</v>
+      </c>
+      <c r="H8" s="20" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="I8" s="17" t="inlineStr">
+        <is>
+          <t>22.7s</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="16" t="inlineStr">
+        <is>
+          <t>ARIMA(1,1,1)</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>5915.22</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>5626.12</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>7813.31</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="I9" s="17" t="inlineStr">
+        <is>
+          <t>8.7s</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal Naive</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on all 300 high-volume groups)</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>5969.34</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>5856.3</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>8924.129999999999</v>
+      </c>
+      <c r="H10" s="20" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="I10" s="17" t="inlineStr">
+        <is>
+          <t>0.04s</t>
+        </is>
+      </c>
+      <c r="J10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="107" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="27" customWidth="1" min="10" max="10"/>
+    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>50 Groups Evaluation Detailed Results Table</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Evaluated on 50 high-volume controlled validation groups | Validation period: 2012-08-17 to 2012-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Scope</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Groups</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Model Parameters</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>WMAE</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>MAE</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>RMSE</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>sMAPE</t>
+        </is>
+      </c>
+      <c r="I4" s="9" t="inlineStr">
+        <is>
+          <t>Runtime</t>
+        </is>
+      </c>
+      <c r="J4" s="9" t="inlineStr">
+        <is>
+          <t>Improvement vs Baseline</t>
+        </is>
+      </c>
+      <c r="K4" s="9" t="inlineStr">
+        <is>
+          <t>Fit Success</t>
+        </is>
+      </c>
+      <c r="L4" s="9" t="inlineStr">
+        <is>
+          <t>Rank</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Holt-Winters</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>50</v>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="n">
         <v>6838.89</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="F5" s="13" t="n">
         <v>6753.86</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="G5" s="13" t="n">
         <v>9852.280000000001</v>
       </c>
-      <c r="F5" s="12" t="n">
-        <v>6.3481</v>
-      </c>
-      <c r="G5" s="12" t="n">
+      <c r="H5" s="14" t="n">
         <v>6.5</v>
       </c>
-      <c r="H5" s="13" t="inlineStr">
+      <c r="I5" s="11" t="inlineStr">
         <is>
           <t>1.37s</t>
         </is>
       </c>
-      <c r="I5" s="13" t="n">
+      <c r="J5" s="15" t="n">
+        <v>32.65</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L5" s="11" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>SARIMA(1,1,0)x(0,1,1,52)</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="n">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D6" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="n">
         <v>7375.57</v>
       </c>
-      <c r="D6" s="15" t="n">
+      <c r="F6" s="19" t="n">
         <v>7465.79</v>
       </c>
-      <c r="E6" s="15" t="n">
+      <c r="G6" s="19" t="n">
         <v>11072.19</v>
       </c>
-      <c r="F6" s="16" t="n">
-        <v>7.0593</v>
-      </c>
-      <c r="G6" s="16" t="n">
+      <c r="H6" s="20" t="n">
         <v>7.31</v>
       </c>
-      <c r="H6" s="17" t="inlineStr">
+      <c r="I6" s="17" t="inlineStr">
         <is>
           <t>62.2s</t>
         </is>
       </c>
-      <c r="I6" s="17" t="n">
+      <c r="J6" s="21" t="n">
+        <v>27.37</v>
+      </c>
+      <c r="K6" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L6" s="17" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>ARIMA(1,1,1)</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="n">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D7" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="n">
         <v>9148.290000000001</v>
       </c>
-      <c r="D7" s="15" t="n">
+      <c r="F7" s="19" t="n">
         <v>8670.959999999999</v>
       </c>
-      <c r="E7" s="15" t="n">
+      <c r="G7" s="19" t="n">
         <v>11257.67</v>
       </c>
-      <c r="F7" s="16" t="n">
-        <v>7.8766</v>
-      </c>
-      <c r="G7" s="16" t="n">
+      <c r="H7" s="20" t="n">
         <v>7.93</v>
       </c>
-      <c r="H7" s="17" t="inlineStr">
+      <c r="I7" s="17" t="inlineStr">
         <is>
           <t>0.80s</t>
         </is>
       </c>
-      <c r="I7" s="17" t="n">
+      <c r="J7" s="21" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="K7" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L7" s="17" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Simple Exp Smoothing (SES)</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="n">
+      <c r="B8" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D8" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="n">
         <v>9166.110000000001</v>
       </c>
-      <c r="D8" s="15" t="n">
+      <c r="F8" s="19" t="n">
         <v>8779.459999999999</v>
       </c>
-      <c r="E8" s="15" t="n">
+      <c r="G8" s="19" t="n">
         <v>11333.78</v>
       </c>
-      <c r="F8" s="16" t="n">
-        <v>7.9971</v>
-      </c>
-      <c r="G8" s="16" t="n">
+      <c r="H8" s="20" t="n">
         <v>8.039999999999999</v>
       </c>
-      <c r="H8" s="17" t="inlineStr">
+      <c r="I8" s="17" t="inlineStr">
         <is>
           <t>1.99s</t>
         </is>
       </c>
-      <c r="I8" s="17" t="n">
+      <c r="J8" s="21" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="K8" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Holt's Linear Trend</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>Advanced Statistical</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="n">
+      <c r="B9" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E9" s="19" t="n">
         <v>9327.07</v>
       </c>
-      <c r="D9" s="15" t="n">
+      <c r="F9" s="19" t="n">
         <v>8889.629999999999</v>
       </c>
-      <c r="E9" s="15" t="n">
+      <c r="G9" s="19" t="n">
         <v>11473.64</v>
       </c>
-      <c r="F9" s="16" t="n">
-        <v>8.047499999999999</v>
-      </c>
-      <c r="G9" s="16" t="n">
+      <c r="H9" s="20" t="n">
         <v>8.119999999999999</v>
       </c>
-      <c r="H9" s="17" t="inlineStr">
+      <c r="I9" s="17" t="inlineStr">
         <is>
           <t>0.46s</t>
         </is>
       </c>
-      <c r="I9" s="17" t="n">
+      <c r="J9" s="21" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="K9" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L9" s="17" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Seasonal Naive</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>Baseline Model</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="n">
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D10" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on all 50 high-volume groups)</t>
+        </is>
+      </c>
+      <c r="E10" s="19" t="n">
         <v>10154.41</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="F10" s="19" t="n">
         <v>9921.17</v>
       </c>
-      <c r="E10" s="15" t="n">
+      <c r="G10" s="19" t="n">
         <v>14704.32</v>
       </c>
-      <c r="F10" s="16" t="n">
-        <v>9.2912</v>
-      </c>
-      <c r="G10" s="16" t="n">
+      <c r="H10" s="20" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="H10" s="17" t="inlineStr">
+      <c r="I10" s="17" t="inlineStr">
         <is>
           <t>0.01s</t>
         </is>
       </c>
-      <c r="I10" s="17" t="n">
+      <c r="J10" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L10" s="17" t="n">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update results/model_comparison_report.xlsx with 9 machine learning model results, styling highlights, and key summary findings
</commit_message>
<xml_diff>
--- a/results/model_comparison_report.xlsx
+++ b/results/model_comparison_report.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="+0.00%;-0.00%;0.00%"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -94,11 +94,17 @@
     </font>
     <font>
       <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Segoe UI"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +121,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
         <bgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+        <bgColor rgb="00DDEBF7"/>
       </patternFill>
     </fill>
   </fills>
@@ -150,7 +162,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -205,10 +217,28 @@
     <xf numFmtId="165" fontId="11" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="12" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="13" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -674,42 +704,42 @@
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>1. Holt-Winters (Triple Exponential Smoothing) is the undisputed winner across all three evaluation datasets.</t>
+          <t>1. Machine Learning models (Random Forest, LightGBM, XGBoost) achieve the lowest overall errors on the Full Dataset.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>2. On the full dataset (All Groups), Holt-Winters reduced WMAE by 17.1% relative to the Seasonal Naïve baseline.</t>
+          <t>2. Random Forest is the overall champion, reducing WMAE to $1,292.53 (a 24.99% improvement vs. Seasonal Naïve baseline).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>3. Models with explicit seasonal components (Holt-Winters, SARIMA, Seasonal Naïve) vastly outperform non-seasonal models.</t>
+          <t>3. LightGBM is the runner-up and highly efficient, achieving a WMAE of $1,304.36 in only 17.8 seconds of training.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>4. Damped trend parameters prevent Holt-Winters from over-projecting recent sales trends over the 12-week horizon.</t>
+          <t>4. Among statistical approaches, Holt-Winters remains the best-performing model (WMAE $1,427.69, a 17.15% improvement).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>5. Running SARIMAX with simple_differencing=False successfully integrates predictions back to level sales space.</t>
+          <t>5. Tree-based ML models successfully capture complex interactions (lags, rolling stats, holiday effects) without explicit seasonal parameters.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>6. Parallel execution using n_jobs=-1 utilizes all 16 CPU cores, completing 300 group evaluations in just 17.2 seconds.</t>
+          <t>6. Simple Linear Regression and Neural Networks (MLP, ANN) lag behind because they struggle to model high-frequency seasonality robustly.</t>
         </is>
       </c>
     </row>
@@ -724,7 +754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L25"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -820,7 +850,7 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -833,32 +863,32 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+          <t>n_estimators=100, max_depth=15, min_samples_split=5</t>
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>1427.69</v>
+        <v>1292.53</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>1422.5</v>
+        <v>1230.3</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>3130.43</v>
+        <v>2560.28</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>23.71</v>
+        <v>17.59</v>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>33.4 min (2006s)</t>
+          <t>1.9 min (115.6s)</t>
         </is>
       </c>
       <c r="J5" s="15" t="n">
-        <v>17.15</v>
+        <v>24.99</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L5" s="11" t="n">
@@ -868,7 +898,7 @@
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
@@ -881,32 +911,32 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+          <t>objective='regression_l1', n_estimators=500, learning_rate=0.05, num_leaves=31, n_jobs=1</t>
         </is>
       </c>
       <c r="E6" s="19" t="n">
-        <v>1494.19</v>
+        <v>1304.36</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>1495.93</v>
+        <v>1227.3</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>3189.19</v>
+        <v>2672.45</v>
       </c>
       <c r="H6" s="20" t="n">
-        <v>24.42</v>
+        <v>17.64</v>
       </c>
       <c r="I6" s="17" t="inlineStr">
         <is>
-          <t>57.3 min (3436s)</t>
+          <t>17.8s</t>
         </is>
       </c>
       <c r="J6" s="21" t="n">
-        <v>13.29</v>
+        <v>24.3</v>
       </c>
       <c r="K6" s="16" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L6" s="17" t="n">
@@ -916,7 +946,7 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Seasonal Naive (Subset)</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
@@ -929,32 +959,32 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>period=52 (evaluated on eligible groups with &gt;= 104 weeks history)</t>
+          <t>n_estimators=100, max_depth=6, learning_rate=0.1, n_jobs=-1</t>
         </is>
       </c>
       <c r="E7" s="19" t="n">
-        <v>1714.9</v>
+        <v>1357.43</v>
       </c>
       <c r="F7" s="19" t="n">
-        <v>1689.93</v>
+        <v>1275.75</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>3638.77</v>
+        <v>2821.77</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>23.35</v>
+        <v>21.91</v>
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>2.9s</t>
         </is>
       </c>
       <c r="J7" s="21" t="n">
-        <v>0.48</v>
+        <v>21.22</v>
       </c>
       <c r="K7" s="16" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L7" s="17" t="n">
@@ -964,7 +994,7 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Seasonal Naive (Full)</t>
+          <t>Ensemble (RF+XGB+LGBM+MLP)</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
@@ -977,28 +1007,28 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>period=52 (evaluated on all 3,084 groups)</t>
+          <t>Uniform average of Random Forest, XGBoost, LightGBM, and MLP predictions</t>
         </is>
       </c>
       <c r="E8" s="19" t="n">
-        <v>1723.13</v>
+        <v>1419.14</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>1698.02</v>
+        <v>1298.52</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>3658.17</v>
+        <v>2629.27</v>
       </c>
       <c r="H8" s="20" t="n">
-        <v>23.46</v>
+        <v>27.03</v>
       </c>
       <c r="I8" s="17" t="inlineStr">
         <is>
-          <t>0.13s</t>
-        </is>
-      </c>
-      <c r="J8" s="22" t="n">
-        <v>0</v>
+          <t>2.5 min (152.1s)</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>17.64</v>
       </c>
       <c r="K8" s="16" t="inlineStr">
         <is>
@@ -1010,57 +1040,57 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Simple Exp Smoothing (SES)</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Holt-Winters</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>Full Dataset</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="24" t="n">
         <v>3084</v>
       </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>initialization_method='estimated' (optimized alpha)</t>
-        </is>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>2143.17</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>2156.63</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>4800.22</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>26.41</v>
-      </c>
-      <c r="I9" s="17" t="inlineStr">
-        <is>
-          <t>33.8 min (2029s)</t>
-        </is>
-      </c>
-      <c r="J9" s="23" t="n">
-        <v>-24.38</v>
-      </c>
-      <c r="K9" s="16" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>1427.69</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>1422.5</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>3130.43</v>
+      </c>
+      <c r="H9" s="26" t="n">
+        <v>23.71</v>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>33.4 min (2006s)</t>
+        </is>
+      </c>
+      <c r="J9" s="27" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="K9" s="22" t="inlineStr">
         <is>
           <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
         </is>
       </c>
-      <c r="L9" s="17" t="n">
+      <c r="L9" s="23" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Holt's Linear Trend</t>
+          <t>GBRT</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
@@ -1073,32 +1103,32 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+          <t>n_estimators=100, max_depth=4, learning_rate=0.1</t>
         </is>
       </c>
       <c r="E10" s="19" t="n">
-        <v>2155.95</v>
+        <v>1457.42</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>2166.05</v>
+        <v>1359.67</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>5261.12</v>
+        <v>2753.77</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>27.01</v>
+        <v>24.43</v>
       </c>
       <c r="I10" s="17" t="inlineStr">
         <is>
-          <t>32.9 min (1974s)</t>
-        </is>
-      </c>
-      <c r="J10" s="23" t="n">
-        <v>-25.12</v>
+          <t>9.0 min (540.2s)</t>
+        </is>
+      </c>
+      <c r="J10" s="21" t="n">
+        <v>15.42</v>
       </c>
       <c r="K10" s="16" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L10" s="17" t="n">
@@ -1108,7 +1138,7 @@
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>ARIMA(1,1,1)</t>
+          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
@@ -1121,28 +1151,28 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>order=(1,1,1) fit per group</t>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>2210.61</v>
+        <v>1494.19</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>2197.86</v>
+        <v>1495.93</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>4920.17</v>
+        <v>3189.19</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>26.33</v>
+        <v>24.42</v>
       </c>
       <c r="I11" s="17" t="inlineStr">
         <is>
-          <t>35.5 min (2131s)</t>
-        </is>
-      </c>
-      <c r="J11" s="23" t="n">
-        <v>-28.29</v>
+          <t>57.3 min (3436s)</t>
+        </is>
+      </c>
+      <c r="J11" s="21" t="n">
+        <v>13.29</v>
       </c>
       <c r="K11" s="16" t="inlineStr">
         <is>
@@ -1156,7 +1186,7 @@
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Naive</t>
+          <t>Seasonal Naive (Subset)</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
@@ -1169,32 +1199,32 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>period=1 (uses final week's sales value as static forecast)</t>
+          <t>period=52 (evaluated on eligible groups with &gt;= 104 weeks history)</t>
         </is>
       </c>
       <c r="E12" s="19" t="n">
-        <v>2241.28</v>
+        <v>1714.9</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>2308.47</v>
+        <v>1689.93</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>5080.3</v>
+        <v>3638.77</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>28.25</v>
+        <v>23.35</v>
       </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
           <t>0.16s</t>
         </is>
       </c>
-      <c r="J12" s="23" t="n">
-        <v>-30.07</v>
+      <c r="J12" s="21" t="n">
+        <v>0.48</v>
       </c>
       <c r="K12" s="16" t="inlineStr">
         <is>
-          <t>100.0% (3084/3084) Success</t>
+          <t>91.96% (2836/3084) Success</t>
         </is>
       </c>
       <c r="L12" s="17" t="n">
@@ -1204,7 +1234,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Historical Mean</t>
+          <t>Seasonal Naive (Full)</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
@@ -1217,28 +1247,28 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>static average calculated per group</t>
+          <t>period=52 (evaluated on all 3,084 groups)</t>
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>2524.38</v>
+        <v>1723.13</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>2425.44</v>
+        <v>1698.02</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>4953.47</v>
+        <v>3658.17</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>29.2</v>
+        <v>23.46</v>
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>0.03s</t>
-        </is>
-      </c>
-      <c r="J13" s="23" t="n">
-        <v>-46.5</v>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n">
+        <v>0</v>
       </c>
       <c r="K13" s="16" t="inlineStr">
         <is>
@@ -1250,99 +1280,99 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>Holt-Winters</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>300 High-Volume</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="n">
-        <v>300</v>
-      </c>
-      <c r="D14" s="10" t="inlineStr">
-        <is>
-          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
-        </is>
-      </c>
-      <c r="E14" s="13" t="n">
-        <v>4538.4</v>
-      </c>
-      <c r="F14" s="13" t="n">
-        <v>4557.37</v>
-      </c>
-      <c r="G14" s="13" t="n">
-        <v>6930.41</v>
-      </c>
-      <c r="H14" s="14" t="n">
-        <v>7.49</v>
-      </c>
-      <c r="I14" s="11" t="inlineStr">
-        <is>
-          <t>17.2s</t>
-        </is>
-      </c>
-      <c r="J14" s="15" t="n">
-        <v>23.97</v>
-      </c>
-      <c r="K14" s="10" t="inlineStr">
-        <is>
-          <t>100.0% (300/300) Success</t>
-        </is>
-      </c>
-      <c r="L14" s="11" t="n">
-        <v>1</v>
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>n_neighbors=10, weights='distance'</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>1782.23</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>1731.91</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>3200.61</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>13.6s</t>
+        </is>
+      </c>
+      <c r="J14" s="29" t="n">
+        <v>-3.43</v>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L14" s="17" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+          <t>Linear Regression</t>
         </is>
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>300 High-Volume</t>
+          <t>Full Dataset</t>
         </is>
       </c>
       <c r="C15" s="18" t="n">
-        <v>300</v>
+        <v>3084</v>
       </c>
       <c r="D15" s="16" t="inlineStr">
         <is>
-          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+          <t>OLS regression with lag and rolling features</t>
         </is>
       </c>
       <c r="E15" s="19" t="n">
-        <v>4721.37</v>
+        <v>1830.56</v>
       </c>
       <c r="F15" s="19" t="n">
-        <v>4761.32</v>
+        <v>1743.58</v>
       </c>
       <c r="G15" s="19" t="n">
-        <v>7166.81</v>
+        <v>3465.22</v>
       </c>
       <c r="H15" s="20" t="n">
-        <v>7.82</v>
+        <v>41.97</v>
       </c>
       <c r="I15" s="17" t="inlineStr">
         <is>
-          <t>168.4s</t>
-        </is>
-      </c>
-      <c r="J15" s="21" t="n">
-        <v>20.91</v>
+          <t>1.7s</t>
+        </is>
+      </c>
+      <c r="J15" s="29" t="n">
+        <v>-6.23</v>
       </c>
       <c r="K15" s="16" t="inlineStr">
         <is>
-          <t>100.0% (300/300) Success</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L15" s="17" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -1353,11 +1383,11 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>300 High-Volume</t>
+          <t>Full Dataset</t>
         </is>
       </c>
       <c r="C16" s="18" t="n">
-        <v>300</v>
+        <v>3084</v>
       </c>
       <c r="D16" s="16" t="inlineStr">
         <is>
@@ -1365,32 +1395,32 @@
         </is>
       </c>
       <c r="E16" s="19" t="n">
-        <v>5842.2</v>
+        <v>2143.17</v>
       </c>
       <c r="F16" s="19" t="n">
-        <v>5639.89</v>
+        <v>2156.63</v>
       </c>
       <c r="G16" s="19" t="n">
-        <v>7977.69</v>
+        <v>4800.22</v>
       </c>
       <c r="H16" s="20" t="n">
-        <v>8.859999999999999</v>
+        <v>26.41</v>
       </c>
       <c r="I16" s="17" t="inlineStr">
         <is>
-          <t>29.5s</t>
-        </is>
-      </c>
-      <c r="J16" s="21" t="n">
-        <v>2.13</v>
+          <t>33.8 min (2029s)</t>
+        </is>
+      </c>
+      <c r="J16" s="29" t="n">
+        <v>-24.38</v>
       </c>
       <c r="K16" s="16" t="inlineStr">
         <is>
-          <t>100.0% (300/300) Success</t>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
         </is>
       </c>
       <c r="L16" s="17" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="17">
@@ -1401,11 +1431,11 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>300 High-Volume</t>
+          <t>Full Dataset</t>
         </is>
       </c>
       <c r="C17" s="18" t="n">
-        <v>300</v>
+        <v>3084</v>
       </c>
       <c r="D17" s="16" t="inlineStr">
         <is>
@@ -1413,32 +1443,32 @@
         </is>
       </c>
       <c r="E17" s="19" t="n">
-        <v>5882.53</v>
+        <v>2155.95</v>
       </c>
       <c r="F17" s="19" t="n">
-        <v>5679.11</v>
+        <v>2166.05</v>
       </c>
       <c r="G17" s="19" t="n">
-        <v>8026.3</v>
+        <v>5261.12</v>
       </c>
       <c r="H17" s="20" t="n">
-        <v>8.91</v>
+        <v>27.01</v>
       </c>
       <c r="I17" s="17" t="inlineStr">
         <is>
-          <t>22.7s</t>
-        </is>
-      </c>
-      <c r="J17" s="21" t="n">
-        <v>1.45</v>
+          <t>32.9 min (1974s)</t>
+        </is>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>-25.12</v>
       </c>
       <c r="K17" s="16" t="inlineStr">
         <is>
-          <t>100.0% (300/300) Success</t>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
         </is>
       </c>
       <c r="L17" s="17" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18">
@@ -1449,11 +1479,11 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>300 High-Volume</t>
+          <t>Full Dataset</t>
         </is>
       </c>
       <c r="C18" s="18" t="n">
-        <v>300</v>
+        <v>3084</v>
       </c>
       <c r="D18" s="16" t="inlineStr">
         <is>
@@ -1461,367 +1491,799 @@
         </is>
       </c>
       <c r="E18" s="19" t="n">
-        <v>5915.22</v>
+        <v>2210.61</v>
       </c>
       <c r="F18" s="19" t="n">
-        <v>5626.12</v>
+        <v>2197.86</v>
       </c>
       <c r="G18" s="19" t="n">
-        <v>7813.31</v>
+        <v>4920.17</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>8.85</v>
+        <v>26.33</v>
       </c>
       <c r="I18" s="17" t="inlineStr">
         <is>
-          <t>8.7s</t>
-        </is>
-      </c>
-      <c r="J18" s="21" t="n">
-        <v>0.91</v>
+          <t>35.5 min (2131s)</t>
+        </is>
+      </c>
+      <c r="J18" s="29" t="n">
+        <v>-28.29</v>
       </c>
       <c r="K18" s="16" t="inlineStr">
         <is>
-          <t>100.0% (300/300) Success</t>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
         </is>
       </c>
       <c r="L18" s="17" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Seasonal Naive</t>
+          <t>Naive</t>
         </is>
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>300 High-Volume</t>
+          <t>Full Dataset</t>
         </is>
       </c>
       <c r="C19" s="18" t="n">
-        <v>300</v>
+        <v>3084</v>
       </c>
       <c r="D19" s="16" t="inlineStr">
         <is>
-          <t>period=52 (evaluated on all 300 high-volume groups)</t>
+          <t>period=1 (uses final week's sales value as static forecast)</t>
         </is>
       </c>
       <c r="E19" s="19" t="n">
-        <v>5969.34</v>
+        <v>2241.28</v>
       </c>
       <c r="F19" s="19" t="n">
-        <v>5856.3</v>
+        <v>2308.47</v>
       </c>
       <c r="G19" s="19" t="n">
-        <v>8924.129999999999</v>
+        <v>5080.3</v>
       </c>
       <c r="H19" s="20" t="n">
-        <v>9.07</v>
+        <v>28.25</v>
       </c>
       <c r="I19" s="17" t="inlineStr">
         <is>
-          <t>0.04s</t>
-        </is>
-      </c>
-      <c r="J19" s="22" t="n">
-        <v>0</v>
+          <t>0.16s</t>
+        </is>
+      </c>
+      <c r="J19" s="29" t="n">
+        <v>-30.07</v>
       </c>
       <c r="K19" s="16" t="inlineStr">
         <is>
-          <t>100.0% (300/300) Success</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L19" s="17" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>Holt-Winters</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>50 High-Volume</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="n">
-        <v>50</v>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
-        </is>
-      </c>
-      <c r="E20" s="13" t="n">
-        <v>6838.89</v>
-      </c>
-      <c r="F20" s="13" t="n">
-        <v>6753.86</v>
-      </c>
-      <c r="G20" s="13" t="n">
-        <v>9852.280000000001</v>
-      </c>
-      <c r="H20" s="14" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="I20" s="11" t="inlineStr">
-        <is>
-          <t>1.37s</t>
-        </is>
-      </c>
-      <c r="J20" s="15" t="n">
-        <v>32.65</v>
-      </c>
-      <c r="K20" s="10" t="inlineStr">
-        <is>
-          <t>100.0% (50/50) Success</t>
-        </is>
-      </c>
-      <c r="L20" s="11" t="n">
-        <v>1</v>
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>ANN</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>PyTorch Feed-Forward network with MSE loss</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>2460.02</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>2406.54</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>3622.35</v>
+      </c>
+      <c r="H20" s="20" t="n">
+        <v>45.77</v>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>61.1s</t>
+        </is>
+      </c>
+      <c r="J20" s="29" t="n">
+        <v>-42.76</v>
+      </c>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>16</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="16" t="inlineStr">
         <is>
-          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+          <t>Historical Mean</t>
         </is>
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>50 High-Volume</t>
+          <t>Full Dataset</t>
         </is>
       </c>
       <c r="C21" s="18" t="n">
-        <v>50</v>
+        <v>3084</v>
       </c>
       <c r="D21" s="16" t="inlineStr">
         <is>
-          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+          <t>static average calculated per group</t>
         </is>
       </c>
       <c r="E21" s="19" t="n">
-        <v>7375.57</v>
+        <v>2524.38</v>
       </c>
       <c r="F21" s="19" t="n">
-        <v>7465.79</v>
+        <v>2425.44</v>
       </c>
       <c r="G21" s="19" t="n">
-        <v>11072.19</v>
+        <v>4953.47</v>
       </c>
       <c r="H21" s="20" t="n">
-        <v>7.31</v>
+        <v>29.2</v>
       </c>
       <c r="I21" s="17" t="inlineStr">
         <is>
-          <t>62.2s</t>
-        </is>
-      </c>
-      <c r="J21" s="21" t="n">
-        <v>27.37</v>
+          <t>0.03s</t>
+        </is>
+      </c>
+      <c r="J21" s="29" t="n">
+        <v>-46.5</v>
       </c>
       <c r="K21" s="16" t="inlineStr">
         <is>
-          <t>100.0% (50/50) Success</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L21" s="17" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="16" t="inlineStr">
         <is>
-          <t>ARIMA(1,1,1)</t>
+          <t>MLP</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>50 High-Volume</t>
+          <t>Full Dataset</t>
         </is>
       </c>
       <c r="C22" s="18" t="n">
-        <v>50</v>
+        <v>3084</v>
       </c>
       <c r="D22" s="16" t="inlineStr">
         <is>
-          <t>order=(1,1,1) fit per group</t>
+          <t>hidden_layer_sizes=(64, 32), max_iter=20</t>
         </is>
       </c>
       <c r="E22" s="19" t="n">
-        <v>9148.290000000001</v>
+        <v>2592.14</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>8670.959999999999</v>
+        <v>2132.64</v>
       </c>
       <c r="G22" s="19" t="n">
-        <v>11257.67</v>
+        <v>3521.18</v>
       </c>
       <c r="H22" s="20" t="n">
-        <v>7.93</v>
+        <v>45.6</v>
       </c>
       <c r="I22" s="17" t="inlineStr">
         <is>
-          <t>0.80s</t>
-        </is>
-      </c>
-      <c r="J22" s="21" t="n">
-        <v>9.91</v>
+          <t>30.6s</t>
+        </is>
+      </c>
+      <c r="J22" s="29" t="n">
+        <v>-50.43</v>
       </c>
       <c r="K22" s="16" t="inlineStr">
         <is>
-          <t>100.0% (50/50) Success</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L22" s="17" t="n">
-        <v>3</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
-        <is>
-          <t>Simple Exp Smoothing (SES)</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>50 High-Volume</t>
-        </is>
-      </c>
-      <c r="C23" s="18" t="n">
-        <v>50</v>
-      </c>
-      <c r="D23" s="16" t="inlineStr">
-        <is>
-          <t>initialization_method='estimated' (optimized alpha)</t>
-        </is>
-      </c>
-      <c r="E23" s="19" t="n">
-        <v>9166.110000000001</v>
-      </c>
-      <c r="F23" s="19" t="n">
-        <v>8779.459999999999</v>
-      </c>
-      <c r="G23" s="19" t="n">
-        <v>11333.78</v>
-      </c>
-      <c r="H23" s="20" t="n">
-        <v>8.039999999999999</v>
-      </c>
-      <c r="I23" s="17" t="inlineStr">
-        <is>
-          <t>1.99s</t>
-        </is>
-      </c>
-      <c r="J23" s="21" t="n">
-        <v>9.73</v>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>100.0% (50/50) Success</t>
-        </is>
-      </c>
-      <c r="L23" s="17" t="n">
-        <v>4</v>
+      <c r="A23" s="22" t="inlineStr">
+        <is>
+          <t>Holt-Winters</t>
+        </is>
+      </c>
+      <c r="B23" s="23" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C23" s="24" t="n">
+        <v>300</v>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E23" s="25" t="n">
+        <v>4538.4</v>
+      </c>
+      <c r="F23" s="25" t="n">
+        <v>4557.37</v>
+      </c>
+      <c r="G23" s="25" t="n">
+        <v>6930.41</v>
+      </c>
+      <c r="H23" s="26" t="n">
+        <v>7.49</v>
+      </c>
+      <c r="I23" s="23" t="inlineStr">
+        <is>
+          <t>17.2s</t>
+        </is>
+      </c>
+      <c r="J23" s="27" t="n">
+        <v>23.97</v>
+      </c>
+      <c r="K23" s="22" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L23" s="23" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="16" t="inlineStr">
         <is>
-          <t>Holt's Linear Trend</t>
+          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>50 High-Volume</t>
+          <t>300 High-Volume</t>
         </is>
       </c>
       <c r="C24" s="18" t="n">
-        <v>50</v>
+        <v>300</v>
       </c>
       <c r="D24" s="16" t="inlineStr">
         <is>
-          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
         </is>
       </c>
       <c r="E24" s="19" t="n">
-        <v>9327.07</v>
+        <v>4721.37</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>8889.629999999999</v>
+        <v>4761.32</v>
       </c>
       <c r="G24" s="19" t="n">
-        <v>11473.64</v>
+        <v>7166.81</v>
       </c>
       <c r="H24" s="20" t="n">
-        <v>8.119999999999999</v>
+        <v>7.82</v>
       </c>
       <c r="I24" s="17" t="inlineStr">
         <is>
-          <t>0.46s</t>
+          <t>168.4s</t>
         </is>
       </c>
       <c r="J24" s="21" t="n">
-        <v>8.15</v>
+        <v>20.91</v>
       </c>
       <c r="K24" s="16" t="inlineStr">
         <is>
-          <t>100.0% (50/50) Success</t>
+          <t>100.0% (300/300) Success</t>
         </is>
       </c>
       <c r="L24" s="17" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="16" t="inlineStr">
         <is>
+          <t>Simple Exp Smoothing (SES)</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E25" s="19" t="n">
+        <v>5842.2</v>
+      </c>
+      <c r="F25" s="19" t="n">
+        <v>5639.89</v>
+      </c>
+      <c r="G25" s="19" t="n">
+        <v>7977.69</v>
+      </c>
+      <c r="H25" s="20" t="n">
+        <v>8.859999999999999</v>
+      </c>
+      <c r="I25" s="17" t="inlineStr">
+        <is>
+          <t>29.5s</t>
+        </is>
+      </c>
+      <c r="J25" s="21" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="K25" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L25" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="inlineStr">
+        <is>
+          <t>Holt's Linear Trend</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C26" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E26" s="19" t="n">
+        <v>5882.53</v>
+      </c>
+      <c r="F26" s="19" t="n">
+        <v>5679.11</v>
+      </c>
+      <c r="G26" s="19" t="n">
+        <v>8026.3</v>
+      </c>
+      <c r="H26" s="20" t="n">
+        <v>8.91</v>
+      </c>
+      <c r="I26" s="17" t="inlineStr">
+        <is>
+          <t>22.7s</t>
+        </is>
+      </c>
+      <c r="J26" s="21" t="n">
+        <v>1.45</v>
+      </c>
+      <c r="K26" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L26" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>ARIMA(1,1,1)</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C27" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E27" s="19" t="n">
+        <v>5915.22</v>
+      </c>
+      <c r="F27" s="19" t="n">
+        <v>5626.12</v>
+      </c>
+      <c r="G27" s="19" t="n">
+        <v>7813.31</v>
+      </c>
+      <c r="H27" s="20" t="n">
+        <v>8.85</v>
+      </c>
+      <c r="I27" s="17" t="inlineStr">
+        <is>
+          <t>8.7s</t>
+        </is>
+      </c>
+      <c r="J27" s="21" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="K27" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L27" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="inlineStr">
+        <is>
           <t>Seasonal Naive</t>
         </is>
       </c>
-      <c r="B25" s="17" t="inlineStr">
+      <c r="B28" s="17" t="inlineStr">
+        <is>
+          <t>300 High-Volume</t>
+        </is>
+      </c>
+      <c r="C28" s="18" t="n">
+        <v>300</v>
+      </c>
+      <c r="D28" s="16" t="inlineStr">
+        <is>
+          <t>period=52 (evaluated on all 300 high-volume groups)</t>
+        </is>
+      </c>
+      <c r="E28" s="19" t="n">
+        <v>5969.34</v>
+      </c>
+      <c r="F28" s="19" t="n">
+        <v>5856.3</v>
+      </c>
+      <c r="G28" s="19" t="n">
+        <v>8924.129999999999</v>
+      </c>
+      <c r="H28" s="20" t="n">
+        <v>9.07</v>
+      </c>
+      <c r="I28" s="17" t="inlineStr">
+        <is>
+          <t>0.04s</t>
+        </is>
+      </c>
+      <c r="J28" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="K28" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (300/300) Success</t>
+        </is>
+      </c>
+      <c r="L28" s="17" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="inlineStr">
+        <is>
+          <t>Holt-Winters</t>
+        </is>
+      </c>
+      <c r="B29" s="23" t="inlineStr">
         <is>
           <t>50 High-Volume</t>
         </is>
       </c>
-      <c r="C25" s="18" t="n">
+      <c r="C29" s="24" t="n">
         <v>50</v>
       </c>
-      <c r="D25" s="16" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E29" s="25" t="n">
+        <v>6838.89</v>
+      </c>
+      <c r="F29" s="25" t="n">
+        <v>6753.86</v>
+      </c>
+      <c r="G29" s="25" t="n">
+        <v>9852.280000000001</v>
+      </c>
+      <c r="H29" s="26" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="I29" s="23" t="inlineStr">
+        <is>
+          <t>1.37s</t>
+        </is>
+      </c>
+      <c r="J29" s="27" t="n">
+        <v>32.65</v>
+      </c>
+      <c r="K29" s="22" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L29" s="23" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="16" t="inlineStr">
+        <is>
+          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+        </is>
+      </c>
+      <c r="B30" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D30" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="n">
+        <v>7375.57</v>
+      </c>
+      <c r="F30" s="19" t="n">
+        <v>7465.79</v>
+      </c>
+      <c r="G30" s="19" t="n">
+        <v>11072.19</v>
+      </c>
+      <c r="H30" s="20" t="n">
+        <v>7.31</v>
+      </c>
+      <c r="I30" s="17" t="inlineStr">
+        <is>
+          <t>62.2s</t>
+        </is>
+      </c>
+      <c r="J30" s="21" t="n">
+        <v>27.37</v>
+      </c>
+      <c r="K30" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L30" s="17" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="16" t="inlineStr">
+        <is>
+          <t>ARIMA(1,1,1)</t>
+        </is>
+      </c>
+      <c r="B31" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D31" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E31" s="19" t="n">
+        <v>9148.290000000001</v>
+      </c>
+      <c r="F31" s="19" t="n">
+        <v>8670.959999999999</v>
+      </c>
+      <c r="G31" s="19" t="n">
+        <v>11257.67</v>
+      </c>
+      <c r="H31" s="20" t="n">
+        <v>7.93</v>
+      </c>
+      <c r="I31" s="17" t="inlineStr">
+        <is>
+          <t>0.80s</t>
+        </is>
+      </c>
+      <c r="J31" s="21" t="n">
+        <v>9.91</v>
+      </c>
+      <c r="K31" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L31" s="17" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Simple Exp Smoothing (SES)</t>
+        </is>
+      </c>
+      <c r="B32" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C32" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E32" s="19" t="n">
+        <v>9166.110000000001</v>
+      </c>
+      <c r="F32" s="19" t="n">
+        <v>8779.459999999999</v>
+      </c>
+      <c r="G32" s="19" t="n">
+        <v>11333.78</v>
+      </c>
+      <c r="H32" s="20" t="n">
+        <v>8.039999999999999</v>
+      </c>
+      <c r="I32" s="17" t="inlineStr">
+        <is>
+          <t>1.99s</t>
+        </is>
+      </c>
+      <c r="J32" s="21" t="n">
+        <v>9.73</v>
+      </c>
+      <c r="K32" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L32" s="17" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Holt's Linear Trend</t>
+        </is>
+      </c>
+      <c r="B33" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C33" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E33" s="19" t="n">
+        <v>9327.07</v>
+      </c>
+      <c r="F33" s="19" t="n">
+        <v>8889.629999999999</v>
+      </c>
+      <c r="G33" s="19" t="n">
+        <v>11473.64</v>
+      </c>
+      <c r="H33" s="20" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="I33" s="17" t="inlineStr">
+        <is>
+          <t>0.46s</t>
+        </is>
+      </c>
+      <c r="J33" s="21" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="K33" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (50/50) Success</t>
+        </is>
+      </c>
+      <c r="L33" s="17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Seasonal Naive</t>
+        </is>
+      </c>
+      <c r="B34" s="17" t="inlineStr">
+        <is>
+          <t>50 High-Volume</t>
+        </is>
+      </c>
+      <c r="C34" s="18" t="n">
+        <v>50</v>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
         <is>
           <t>period=52 (evaluated on all 50 high-volume groups)</t>
         </is>
       </c>
-      <c r="E25" s="19" t="n">
+      <c r="E34" s="19" t="n">
         <v>10154.41</v>
       </c>
-      <c r="F25" s="19" t="n">
+      <c r="F34" s="19" t="n">
         <v>9921.17</v>
       </c>
-      <c r="G25" s="19" t="n">
+      <c r="G34" s="19" t="n">
         <v>14704.32</v>
       </c>
-      <c r="H25" s="20" t="n">
+      <c r="H34" s="20" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="I25" s="17" t="inlineStr">
+      <c r="I34" s="17" t="inlineStr">
         <is>
           <t>0.01s</t>
         </is>
       </c>
-      <c r="J25" s="22" t="n">
+      <c r="J34" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="16" t="inlineStr">
+      <c r="K34" s="16" t="inlineStr">
         <is>
           <t>100.0% (50/50) Success</t>
         </is>
       </c>
-      <c r="L25" s="17" t="n">
+      <c r="L34" s="17" t="n">
         <v>6</v>
       </c>
     </row>
@@ -1836,7 +2298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L13"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1932,7 +2394,7 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
-          <t>Holt-Winters</t>
+          <t>Random Forest</t>
         </is>
       </c>
       <c r="B5" s="11" t="inlineStr">
@@ -1945,32 +2407,32 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+          <t>n_estimators=100, max_depth=15, min_samples_split=5</t>
         </is>
       </c>
       <c r="E5" s="13" t="n">
-        <v>1427.69</v>
+        <v>1292.53</v>
       </c>
       <c r="F5" s="13" t="n">
-        <v>1422.5</v>
+        <v>1230.3</v>
       </c>
       <c r="G5" s="13" t="n">
-        <v>3130.43</v>
+        <v>2560.28</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>23.71</v>
+        <v>17.59</v>
       </c>
       <c r="I5" s="11" t="inlineStr">
         <is>
-          <t>33.4 min (2006s)</t>
+          <t>1.9 min (115.6s)</t>
         </is>
       </c>
       <c r="J5" s="15" t="n">
-        <v>17.15</v>
+        <v>24.99</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L5" s="11" t="n">
@@ -1980,7 +2442,7 @@
     <row r="6">
       <c r="A6" s="16" t="inlineStr">
         <is>
-          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
+          <t>LightGBM</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
@@ -1993,32 +2455,32 @@
       </c>
       <c r="D6" s="16" t="inlineStr">
         <is>
-          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
+          <t>objective='regression_l1', n_estimators=500, learning_rate=0.05, num_leaves=31, n_jobs=1</t>
         </is>
       </c>
       <c r="E6" s="19" t="n">
-        <v>1494.19</v>
+        <v>1304.36</v>
       </c>
       <c r="F6" s="19" t="n">
-        <v>1495.93</v>
+        <v>1227.3</v>
       </c>
       <c r="G6" s="19" t="n">
-        <v>3189.19</v>
+        <v>2672.45</v>
       </c>
       <c r="H6" s="20" t="n">
-        <v>24.42</v>
+        <v>17.64</v>
       </c>
       <c r="I6" s="17" t="inlineStr">
         <is>
-          <t>57.3 min (3436s)</t>
+          <t>17.8s</t>
         </is>
       </c>
       <c r="J6" s="21" t="n">
-        <v>13.29</v>
+        <v>24.3</v>
       </c>
       <c r="K6" s="16" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L6" s="17" t="n">
@@ -2028,7 +2490,7 @@
     <row r="7">
       <c r="A7" s="16" t="inlineStr">
         <is>
-          <t>Seasonal Naive (Subset)</t>
+          <t>XGBoost</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
@@ -2041,32 +2503,32 @@
       </c>
       <c r="D7" s="16" t="inlineStr">
         <is>
-          <t>period=52 (evaluated on eligible groups with &gt;= 104 weeks history)</t>
+          <t>n_estimators=100, max_depth=6, learning_rate=0.1, n_jobs=-1</t>
         </is>
       </c>
       <c r="E7" s="19" t="n">
-        <v>1714.9</v>
+        <v>1357.43</v>
       </c>
       <c r="F7" s="19" t="n">
-        <v>1689.93</v>
+        <v>1275.75</v>
       </c>
       <c r="G7" s="19" t="n">
-        <v>3638.77</v>
+        <v>2821.77</v>
       </c>
       <c r="H7" s="20" t="n">
-        <v>23.35</v>
+        <v>21.91</v>
       </c>
       <c r="I7" s="17" t="inlineStr">
         <is>
-          <t>0.16s</t>
+          <t>2.9s</t>
         </is>
       </c>
       <c r="J7" s="21" t="n">
-        <v>0.48</v>
+        <v>21.22</v>
       </c>
       <c r="K7" s="16" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L7" s="17" t="n">
@@ -2076,7 +2538,7 @@
     <row r="8">
       <c r="A8" s="16" t="inlineStr">
         <is>
-          <t>Seasonal Naive (Full)</t>
+          <t>Ensemble (RF+XGB+LGBM+MLP)</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
@@ -2089,28 +2551,28 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>period=52 (evaluated on all 3,084 groups)</t>
+          <t>Uniform average of Random Forest, XGBoost, LightGBM, and MLP predictions</t>
         </is>
       </c>
       <c r="E8" s="19" t="n">
-        <v>1723.13</v>
+        <v>1419.14</v>
       </c>
       <c r="F8" s="19" t="n">
-        <v>1698.02</v>
+        <v>1298.52</v>
       </c>
       <c r="G8" s="19" t="n">
-        <v>3658.17</v>
+        <v>2629.27</v>
       </c>
       <c r="H8" s="20" t="n">
-        <v>23.46</v>
+        <v>27.03</v>
       </c>
       <c r="I8" s="17" t="inlineStr">
         <is>
-          <t>0.13s</t>
-        </is>
-      </c>
-      <c r="J8" s="22" t="n">
-        <v>0</v>
+          <t>2.5 min (152.1s)</t>
+        </is>
+      </c>
+      <c r="J8" s="21" t="n">
+        <v>17.64</v>
       </c>
       <c r="K8" s="16" t="inlineStr">
         <is>
@@ -2122,57 +2584,57 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
-        <is>
-          <t>Simple Exp Smoothing (SES)</t>
-        </is>
-      </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>Holt-Winters</t>
+        </is>
+      </c>
+      <c r="B9" s="23" t="inlineStr">
         <is>
           <t>Full Dataset</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="24" t="n">
         <v>3084</v>
       </c>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>initialization_method='estimated' (optimized alpha)</t>
-        </is>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>2143.17</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>2156.63</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>4800.22</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>26.41</v>
-      </c>
-      <c r="I9" s="17" t="inlineStr">
-        <is>
-          <t>33.8 min (2029s)</t>
-        </is>
-      </c>
-      <c r="J9" s="23" t="n">
-        <v>-24.38</v>
-      </c>
-      <c r="K9" s="16" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
+        <is>
+          <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
+        </is>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>1427.69</v>
+      </c>
+      <c r="F9" s="25" t="n">
+        <v>1422.5</v>
+      </c>
+      <c r="G9" s="25" t="n">
+        <v>3130.43</v>
+      </c>
+      <c r="H9" s="26" t="n">
+        <v>23.71</v>
+      </c>
+      <c r="I9" s="23" t="inlineStr">
+        <is>
+          <t>33.4 min (2006s)</t>
+        </is>
+      </c>
+      <c r="J9" s="27" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="K9" s="22" t="inlineStr">
         <is>
           <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
         </is>
       </c>
-      <c r="L9" s="17" t="n">
+      <c r="L9" s="23" t="n">
         <v>5</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="16" t="inlineStr">
         <is>
-          <t>Holt's Linear Trend</t>
+          <t>GBRT</t>
         </is>
       </c>
       <c r="B10" s="17" t="inlineStr">
@@ -2185,32 +2647,32 @@
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+          <t>n_estimators=100, max_depth=4, learning_rate=0.1</t>
         </is>
       </c>
       <c r="E10" s="19" t="n">
-        <v>2155.95</v>
+        <v>1457.42</v>
       </c>
       <c r="F10" s="19" t="n">
-        <v>2166.05</v>
+        <v>1359.67</v>
       </c>
       <c r="G10" s="19" t="n">
-        <v>5261.12</v>
+        <v>2753.77</v>
       </c>
       <c r="H10" s="20" t="n">
-        <v>27.01</v>
+        <v>24.43</v>
       </c>
       <c r="I10" s="17" t="inlineStr">
         <is>
-          <t>32.9 min (1974s)</t>
-        </is>
-      </c>
-      <c r="J10" s="23" t="n">
-        <v>-25.12</v>
+          <t>9.0 min (540.2s)</t>
+        </is>
+      </c>
+      <c r="J10" s="21" t="n">
+        <v>15.42</v>
       </c>
       <c r="K10" s="16" t="inlineStr">
         <is>
-          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+          <t>100.0% (3084/3084) Success</t>
         </is>
       </c>
       <c r="L10" s="17" t="n">
@@ -2220,7 +2682,7 @@
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>ARIMA(1,1,1)</t>
+          <t>SARIMA(1,1,0)x(0,1,1,52)</t>
         </is>
       </c>
       <c r="B11" s="17" t="inlineStr">
@@ -2233,28 +2695,28 @@
       </c>
       <c r="D11" s="16" t="inlineStr">
         <is>
-          <t>order=(1,1,1) fit per group</t>
+          <t>order=(1,1,0), seasonal_order=(0,1,1,52), simple_differencing=False (integrated space)</t>
         </is>
       </c>
       <c r="E11" s="19" t="n">
-        <v>2210.61</v>
+        <v>1494.19</v>
       </c>
       <c r="F11" s="19" t="n">
-        <v>2197.86</v>
+        <v>1495.93</v>
       </c>
       <c r="G11" s="19" t="n">
-        <v>4920.17</v>
+        <v>3189.19</v>
       </c>
       <c r="H11" s="20" t="n">
-        <v>26.33</v>
+        <v>24.42</v>
       </c>
       <c r="I11" s="17" t="inlineStr">
         <is>
-          <t>35.5 min (2131s)</t>
-        </is>
-      </c>
-      <c r="J11" s="23" t="n">
-        <v>-28.29</v>
+          <t>57.3 min (3436s)</t>
+        </is>
+      </c>
+      <c r="J11" s="21" t="n">
+        <v>13.29</v>
       </c>
       <c r="K11" s="16" t="inlineStr">
         <is>
@@ -2268,7 +2730,7 @@
     <row r="12">
       <c r="A12" s="16" t="inlineStr">
         <is>
-          <t>Naive</t>
+          <t>Seasonal Naive (Subset)</t>
         </is>
       </c>
       <c r="B12" s="17" t="inlineStr">
@@ -2281,32 +2743,32 @@
       </c>
       <c r="D12" s="16" t="inlineStr">
         <is>
-          <t>period=1 (uses final week's sales value as static forecast)</t>
+          <t>period=52 (evaluated on eligible groups with &gt;= 104 weeks history)</t>
         </is>
       </c>
       <c r="E12" s="19" t="n">
-        <v>2241.28</v>
+        <v>1714.9</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>2308.47</v>
+        <v>1689.93</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>5080.3</v>
+        <v>3638.77</v>
       </c>
       <c r="H12" s="20" t="n">
-        <v>28.25</v>
+        <v>23.35</v>
       </c>
       <c r="I12" s="17" t="inlineStr">
         <is>
           <t>0.16s</t>
         </is>
       </c>
-      <c r="J12" s="23" t="n">
-        <v>-30.07</v>
+      <c r="J12" s="21" t="n">
+        <v>0.48</v>
       </c>
       <c r="K12" s="16" t="inlineStr">
         <is>
-          <t>100.0% (3084/3084) Success</t>
+          <t>91.96% (2836/3084) Success</t>
         </is>
       </c>
       <c r="L12" s="17" t="n">
@@ -2316,7 +2778,7 @@
     <row r="13">
       <c r="A13" s="16" t="inlineStr">
         <is>
-          <t>Historical Mean</t>
+          <t>Seasonal Naive (Full)</t>
         </is>
       </c>
       <c r="B13" s="17" t="inlineStr">
@@ -2329,28 +2791,28 @@
       </c>
       <c r="D13" s="16" t="inlineStr">
         <is>
-          <t>static average calculated per group</t>
+          <t>period=52 (evaluated on all 3,084 groups)</t>
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>2524.38</v>
+        <v>1723.13</v>
       </c>
       <c r="F13" s="19" t="n">
-        <v>2425.44</v>
+        <v>1698.02</v>
       </c>
       <c r="G13" s="19" t="n">
-        <v>4953.47</v>
+        <v>3658.17</v>
       </c>
       <c r="H13" s="20" t="n">
-        <v>29.2</v>
+        <v>23.46</v>
       </c>
       <c r="I13" s="17" t="inlineStr">
         <is>
-          <t>0.03s</t>
-        </is>
-      </c>
-      <c r="J13" s="23" t="n">
-        <v>-46.5</v>
+          <t>0.13s</t>
+        </is>
+      </c>
+      <c r="J13" s="28" t="n">
+        <v>0</v>
       </c>
       <c r="K13" s="16" t="inlineStr">
         <is>
@@ -2359,6 +2821,438 @@
       </c>
       <c r="L13" s="17" t="n">
         <v>9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="inlineStr">
+        <is>
+          <t>KNN</t>
+        </is>
+      </c>
+      <c r="B14" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D14" s="16" t="inlineStr">
+        <is>
+          <t>n_neighbors=10, weights='distance'</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="n">
+        <v>1782.23</v>
+      </c>
+      <c r="F14" s="19" t="n">
+        <v>1731.91</v>
+      </c>
+      <c r="G14" s="19" t="n">
+        <v>3200.61</v>
+      </c>
+      <c r="H14" s="20" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="I14" s="17" t="inlineStr">
+        <is>
+          <t>13.6s</t>
+        </is>
+      </c>
+      <c r="J14" s="29" t="n">
+        <v>-3.43</v>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L14" s="17" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Linear Regression</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D15" s="16" t="inlineStr">
+        <is>
+          <t>OLS regression with lag and rolling features</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="n">
+        <v>1830.56</v>
+      </c>
+      <c r="F15" s="19" t="n">
+        <v>1743.58</v>
+      </c>
+      <c r="G15" s="19" t="n">
+        <v>3465.22</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>41.97</v>
+      </c>
+      <c r="I15" s="17" t="inlineStr">
+        <is>
+          <t>1.7s</t>
+        </is>
+      </c>
+      <c r="J15" s="29" t="n">
+        <v>-6.23</v>
+      </c>
+      <c r="K15" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L15" s="17" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Simple Exp Smoothing (SES)</t>
+        </is>
+      </c>
+      <c r="B16" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D16" s="16" t="inlineStr">
+        <is>
+          <t>initialization_method='estimated' (optimized alpha)</t>
+        </is>
+      </c>
+      <c r="E16" s="19" t="n">
+        <v>2143.17</v>
+      </c>
+      <c r="F16" s="19" t="n">
+        <v>2156.63</v>
+      </c>
+      <c r="G16" s="19" t="n">
+        <v>4800.22</v>
+      </c>
+      <c r="H16" s="20" t="n">
+        <v>26.41</v>
+      </c>
+      <c r="I16" s="17" t="inlineStr">
+        <is>
+          <t>33.8 min (2029s)</t>
+        </is>
+      </c>
+      <c r="J16" s="29" t="n">
+        <v>-24.38</v>
+      </c>
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L16" s="17" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Holt's Linear Trend</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>trend='add', damped_trend=True (optimized alpha, beta, phi)</t>
+        </is>
+      </c>
+      <c r="E17" s="19" t="n">
+        <v>2155.95</v>
+      </c>
+      <c r="F17" s="19" t="n">
+        <v>2166.05</v>
+      </c>
+      <c r="G17" s="19" t="n">
+        <v>5261.12</v>
+      </c>
+      <c r="H17" s="20" t="n">
+        <v>27.01</v>
+      </c>
+      <c r="I17" s="17" t="inlineStr">
+        <is>
+          <t>32.9 min (1974s)</t>
+        </is>
+      </c>
+      <c r="J17" s="29" t="n">
+        <v>-25.12</v>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L17" s="17" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>ARIMA(1,1,1)</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>order=(1,1,1) fit per group</t>
+        </is>
+      </c>
+      <c r="E18" s="19" t="n">
+        <v>2210.61</v>
+      </c>
+      <c r="F18" s="19" t="n">
+        <v>2197.86</v>
+      </c>
+      <c r="G18" s="19" t="n">
+        <v>4920.17</v>
+      </c>
+      <c r="H18" s="20" t="n">
+        <v>26.33</v>
+      </c>
+      <c r="I18" s="17" t="inlineStr">
+        <is>
+          <t>35.5 min (2131s)</t>
+        </is>
+      </c>
+      <c r="J18" s="29" t="n">
+        <v>-28.29</v>
+      </c>
+      <c r="K18" s="16" t="inlineStr">
+        <is>
+          <t>91.96% (2836/3084) Success, 8.04% Short-Series Fallback</t>
+        </is>
+      </c>
+      <c r="L18" s="17" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
+        <is>
+          <t>Naive</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>period=1 (uses final week's sales value as static forecast)</t>
+        </is>
+      </c>
+      <c r="E19" s="19" t="n">
+        <v>2241.28</v>
+      </c>
+      <c r="F19" s="19" t="n">
+        <v>2308.47</v>
+      </c>
+      <c r="G19" s="19" t="n">
+        <v>5080.3</v>
+      </c>
+      <c r="H19" s="20" t="n">
+        <v>28.25</v>
+      </c>
+      <c r="I19" s="17" t="inlineStr">
+        <is>
+          <t>0.16s</t>
+        </is>
+      </c>
+      <c r="J19" s="29" t="n">
+        <v>-30.07</v>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L19" s="17" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
+        <is>
+          <t>ANN</t>
+        </is>
+      </c>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>PyTorch Feed-Forward network with MSE loss</t>
+        </is>
+      </c>
+      <c r="E20" s="19" t="n">
+        <v>2460.02</v>
+      </c>
+      <c r="F20" s="19" t="n">
+        <v>2406.54</v>
+      </c>
+      <c r="G20" s="19" t="n">
+        <v>3622.35</v>
+      </c>
+      <c r="H20" s="20" t="n">
+        <v>45.77</v>
+      </c>
+      <c r="I20" s="17" t="inlineStr">
+        <is>
+          <t>61.1s</t>
+        </is>
+      </c>
+      <c r="J20" s="29" t="n">
+        <v>-42.76</v>
+      </c>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L20" s="17" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
+        <is>
+          <t>Historical Mean</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D21" s="16" t="inlineStr">
+        <is>
+          <t>static average calculated per group</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>2524.38</v>
+      </c>
+      <c r="F21" s="19" t="n">
+        <v>2425.44</v>
+      </c>
+      <c r="G21" s="19" t="n">
+        <v>4953.47</v>
+      </c>
+      <c r="H21" s="20" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="I21" s="17" t="inlineStr">
+        <is>
+          <t>0.03s</t>
+        </is>
+      </c>
+      <c r="J21" s="29" t="n">
+        <v>-46.5</v>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L21" s="17" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>MLP</t>
+        </is>
+      </c>
+      <c r="B22" s="17" t="inlineStr">
+        <is>
+          <t>Full Dataset</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="n">
+        <v>3084</v>
+      </c>
+      <c r="D22" s="16" t="inlineStr">
+        <is>
+          <t>hidden_layer_sizes=(64, 32), max_iter=20</t>
+        </is>
+      </c>
+      <c r="E22" s="19" t="n">
+        <v>2592.14</v>
+      </c>
+      <c r="F22" s="19" t="n">
+        <v>2132.64</v>
+      </c>
+      <c r="G22" s="19" t="n">
+        <v>3521.18</v>
+      </c>
+      <c r="H22" s="20" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I22" s="17" t="inlineStr">
+        <is>
+          <t>30.6s</t>
+        </is>
+      </c>
+      <c r="J22" s="29" t="n">
+        <v>-50.43</v>
+      </c>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>100.0% (3084/3084) Success</t>
+        </is>
+      </c>
+      <c r="L22" s="17" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -2466,50 +3360,50 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Holt-Winters</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>300 High-Volume</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="24" t="n">
         <v>300</v>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="25" t="n">
         <v>4538.4</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="25" t="n">
         <v>4557.37</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="25" t="n">
         <v>6930.41</v>
       </c>
-      <c r="H5" s="14" t="n">
+      <c r="H5" s="26" t="n">
         <v>7.49</v>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="I5" s="23" t="inlineStr">
         <is>
           <t>17.2s</t>
         </is>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="J5" s="27" t="n">
         <v>23.97</v>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="K5" s="22" t="inlineStr">
         <is>
           <t>100.0% (300/300) Success</t>
         </is>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="23" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2741,7 +3635,7 @@
           <t>0.04s</t>
         </is>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="28" t="n">
         <v>0</v>
       </c>
       <c r="K10" s="16" t="inlineStr">
@@ -2858,50 +3752,50 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="22" t="inlineStr">
         <is>
           <t>Holt-Winters</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>50 High-Volume</t>
         </is>
       </c>
-      <c r="C5" s="12" t="n">
+      <c r="C5" s="24" t="n">
         <v>50</v>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="D5" s="22" t="inlineStr">
         <is>
           <t>trend='add', seasonal='add', seasonal_periods=52, damped_trend=True (optimized alpha, beta, gamma, phi)</t>
         </is>
       </c>
-      <c r="E5" s="13" t="n">
+      <c r="E5" s="25" t="n">
         <v>6838.89</v>
       </c>
-      <c r="F5" s="13" t="n">
+      <c r="F5" s="25" t="n">
         <v>6753.86</v>
       </c>
-      <c r="G5" s="13" t="n">
+      <c r="G5" s="25" t="n">
         <v>9852.280000000001</v>
       </c>
-      <c r="H5" s="14" t="n">
+      <c r="H5" s="26" t="n">
         <v>6.5</v>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="I5" s="23" t="inlineStr">
         <is>
           <t>1.37s</t>
         </is>
       </c>
-      <c r="J5" s="15" t="n">
+      <c r="J5" s="27" t="n">
         <v>32.65</v>
       </c>
-      <c r="K5" s="10" t="inlineStr">
+      <c r="K5" s="22" t="inlineStr">
         <is>
           <t>100.0% (50/50) Success</t>
         </is>
       </c>
-      <c r="L5" s="11" t="n">
+      <c r="L5" s="23" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3133,7 +4027,7 @@
           <t>0.01s</t>
         </is>
       </c>
-      <c r="J10" s="22" t="n">
+      <c r="J10" s="28" t="n">
         <v>0</v>
       </c>
       <c r="K10" s="16" t="inlineStr">

</xml_diff>